<commit_message>
Update 10 July 2025
Districts geojson has manual edits to match Capex
</commit_message>
<xml_diff>
--- a/data/TCPD/2.interim/Matching -COncordance Table.xlsx
+++ b/data/TCPD/2.interim/Matching -COncordance Table.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e46a4301436fbcaf/Kalyan/KK-Python/Kalyan-Jupyter-Notebooks/data/TCPD/2.interim/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{900A9638-2D17-9E45-A366-14213E8A916F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{73BD055A-9D31-6748-A6F1-C670B1F26774}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{900A9638-2D17-9E45-A366-14213E8A916F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2C31642B-685A-B74F-8DCD-CF57963467F6}"/>
   <bookViews>
-    <workbookView xWindow="1480" yWindow="1740" windowWidth="27240" windowHeight="15400" xr2:uid="{24D9D4F4-F069-7F48-9941-DD9973D08A06}"/>
+    <workbookView xWindow="7640" yWindow="2420" windowWidth="27240" windowHeight="15400" xr2:uid="{24D9D4F4-F069-7F48-9941-DD9973D08A06}"/>
   </bookViews>
   <sheets>
-    <sheet name="Field Names" sheetId="1" r:id="rId1"/>
+    <sheet name="IAS Variable Names" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>

</xml_diff>